<commit_message>
Trim trailing whitespace from two spreadsheet names
Now that Excel has released the file, the trim that kept getting overwritten
has been applied: an output called 'Total Available Water ' and a sensor called
'... Soil Temperature Sensor (200TS) ' both carried a trailing space, which
made them awkward to match by hand and easy to mistype.
</commit_message>
<xml_diff>
--- a/data/sensor_configuration_v2.xlsx
+++ b/data/sensor_configuration_v2.xlsx
@@ -992,7 +992,7 @@
       <c r="A10" s="24" t="n"/>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Total Available Water </t>
+          <t>Total Available Water</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Irrometer Watermark (200SS) combined with Irrometer Soil Temperature Sensor (200TS) </t>
+          <t>Irrometer Watermark (200SS) combined with Irrometer Soil Temperature Sensor (200TS)</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">

</xml_diff>

<commit_message>
make the user guide build on a minimal latex install
it needed tcolorbox, titlesec, fancyhdr, enumitem and parskip, none of which
ship with basictex, so a fresh install would have failed on the first missing
package after the person had already installed latex.

it now needs only geometry, xcolor and hyperref, which every distribution has.
the note and caution boxes are built from core latex with a savebox and
fcolorbox, list spacing uses the defaults, and the running header is gone. the
content is unchanged.

the readme now says how to install latex in the first place, since pdflatex is
not on macos by default.
</commit_message>
<xml_diff>
--- a/data/sensor_configuration_v2.xlsx
+++ b/data/sensor_configuration_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fernandolaguna/Desktop/Low-Cost-Water-Tech/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE5DCCCB-5358-2D4C-B25D-14E28B468320}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C02482C7-CBB6-BC4C-A700-02C4A10995BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sensors" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="452" uniqueCount="260">
   <si>
     <t>sensor_name</t>
   </si>
@@ -801,6 +801,9 @@
   </si>
   <si>
     <t>Displays the state at which the soils seems to be for the Watermark sensors</t>
+  </si>
+  <si>
+    <t>The downward movement of water infiltrating through the soil.</t>
   </si>
 </sst>
 </file>
@@ -1549,7 +1552,9 @@
         <v>59</v>
       </c>
       <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
+      <c r="D9" s="3" t="s">
+        <v>259</v>
+      </c>
       <c r="E9" s="3" t="s">
         <v>37</v>
       </c>

</xml_diff>